<commit_message>
Update QUESTIONS.xlsx, images, Scheduled sending message based on client feedback
</commit_message>
<xml_diff>
--- a/Quizbot/data/INTRO.xlsx
+++ b/Quizbot/data/INTRO.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\++My Codes\Web Develop\Telegam_Bale Bot\Keramat_Quizbot2\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\++My Codes\Web Develop\Telegam_Bale Bot\Keramat_Quizbot2\Quizbot\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02FD61E2-7AC0-45E9-B9F9-9AABBB772D34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3201E86-7601-4A63-B636-17E273D21A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,9 +51,6 @@
     <t>marital</t>
   </si>
   <si>
-    <t>وضعیت تاهل خودتونو انتخاب کنین.</t>
-  </si>
-  <si>
     <t>single</t>
   </si>
   <si>
@@ -78,9 +75,6 @@
     <t>child_gender</t>
   </si>
   <si>
-    <t>جنسیت فرزندتون چیه؟</t>
-  </si>
-  <si>
     <t>دختر قندعسل</t>
   </si>
   <si>
@@ -103,6 +97,12 @@
   </si>
   <si>
     <t>خانم مجرد هستم</t>
+  </si>
+  <si>
+    <t>جنسیت فرزندتون چیه؟ 👶</t>
+  </si>
+  <si>
+    <t>وضعیت تاهل خودتونو انتخاب کنین💍</t>
   </si>
 </sst>
 </file>
@@ -476,16 +476,16 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
-      </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -493,19 +493,19 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
-        <v>25</v>
-      </c>
-      <c r="D3" t="s">
-        <v>9</v>
-      </c>
       <c r="E3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -513,19 +513,19 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
         <v>10</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>11</v>
       </c>
-      <c r="E4" t="s">
-        <v>12</v>
-      </c>
       <c r="G4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -533,70 +533,70 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" t="s">
         <v>13</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>14</v>
       </c>
-      <c r="E5" t="s">
-        <v>15</v>
-      </c>
       <c r="G5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" t="s">
         <v>16</v>
       </c>
-      <c r="B6" t="s">
+      <c r="F6" t="s">
         <v>17</v>
       </c>
-      <c r="C6" t="s">
-        <v>18</v>
-      </c>
-      <c r="F6" t="s">
-        <v>19</v>
-      </c>
       <c r="G6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>